<commit_message>
paper run 2026-09-22 11:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-22.xlsx
+++ b/reports/2026-09-22.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,6 +601,49 @@
       </c>
       <c r="K4" t="n">
         <v>-4.24</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-22T10:29:01.367556+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F5" t="n">
+        <v>12.76</v>
+      </c>
+      <c r="G5" t="n">
+        <v>22</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.00125</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>9.24</v>
       </c>
     </row>
   </sheetData>
@@ -614,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,7 +679,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -646,7 +689,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -666,7 +709,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="6">
@@ -676,7 +719,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15.82</v>
+        <v>25.06</v>
       </c>
     </row>
     <row r="7">
@@ -686,7 +729,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20.06</v>
+        <v>29.3</v>
       </c>
     </row>
     <row r="8">
@@ -706,7 +749,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4.73</v>
+        <v>6.91</v>
       </c>
     </row>
     <row r="10">
@@ -716,7 +759,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1420.2</v>
+        <v>1429.44</v>
       </c>
     </row>
     <row r="12">
@@ -786,16 +829,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D16" t="n">
-        <v>192.91</v>
+        <v>346.87</v>
       </c>
       <c r="E16" t="n">
-        <v>9.800000000000001</v>
+        <v>19.04</v>
       </c>
     </row>
     <row r="17">
@@ -850,16 +893,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
-        <v>-30.86</v>
+        <v>123.1</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
     </row>
     <row r="21">
@@ -895,16 +938,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D23" t="n">
-        <v>50.1</v>
+        <v>204.06</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
     </row>
     <row r="24">
@@ -940,13 +983,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C26" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D26" t="n">
-        <v>65.28</v>
+        <v>169.4</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -959,16 +1002,16 @@
         </is>
       </c>
       <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n">
         <v>3</v>
       </c>
-      <c r="C27" t="n">
-        <v>2</v>
-      </c>
       <c r="D27" t="n">
-        <v>36.85</v>
+        <v>86.69</v>
       </c>
       <c r="E27" t="n">
-        <v>15.82</v>
+        <v>25.06</v>
       </c>
     </row>
     <row r="29">
@@ -1032,102 +1075,102 @@
         <v>5.56</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>9.24</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>2</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
-        <v>6.02</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>6.02</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>9.800000000000001</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="n">
+        <v>19.04</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>10.26</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1137,169 +1180,249 @@
         <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>9.800000000000001</v>
+        <v>10.26</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>9.800000000000001</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="n">
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
         <v>0</v>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>-4.24</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>2</v>
-      </c>
-      <c r="C45" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" t="n">
-        <v>5.56</v>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>9.24</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" t="n">
-        <v>10.26</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5.56</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>9.24</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C49" t="n">
         <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>5.56</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>0.15–0.20%</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
         <v>10.26</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>5.56</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>9.24</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>10.26</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B53" t="n">
+      <c r="B57" t="n">
         <v>3</v>
       </c>
-      <c r="C53" t="n">
+      <c r="C57" t="n">
         <v>2</v>
       </c>
-      <c r="D53" t="n">
+      <c r="D57" t="n">
         <v>15.82</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>9.24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-22 17:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-22.xlsx
+++ b/reports/2026-09-22.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +644,221 @@
       </c>
       <c r="K5" t="n">
         <v>9.24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-22T12:54:13.711362+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.00127</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-22T14:13:07.353410+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F7" t="n">
+        <v>22</v>
+      </c>
+      <c r="G7" t="n">
+        <v>40</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00112</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-22T14:38:46.205744+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F8" t="n">
+        <v>72.48999999999999</v>
+      </c>
+      <c r="G8" t="n">
+        <v>139.4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.756</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.00102</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>66.91</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-22T14:41:18.443762+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F9" t="n">
+        <v>72.48999999999999</v>
+      </c>
+      <c r="G9" t="n">
+        <v>142.14</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.00135</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>69.65000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-22T15:42:56.740292+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G10" t="n">
+        <v>14</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.00136</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>5.88</v>
       </c>
     </row>
   </sheetData>
@@ -657,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,7 +894,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -689,7 +904,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -709,7 +924,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.75</v>
+        <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="6">
@@ -719,7 +934,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>25.06</v>
+        <v>187.85</v>
       </c>
     </row>
     <row r="7">
@@ -729,7 +944,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29.3</v>
+        <v>192.09</v>
       </c>
     </row>
     <row r="8">
@@ -749,7 +964,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6.91</v>
+        <v>45.3</v>
       </c>
     </row>
     <row r="10">
@@ -759,7 +974,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1429.44</v>
+        <v>1592.23</v>
       </c>
     </row>
     <row r="12">
@@ -810,16 +1025,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>-90.78</v>
+        <v>255.81</v>
       </c>
       <c r="E15" t="n">
-        <v>6.02</v>
+        <v>99.55</v>
       </c>
     </row>
     <row r="16">
@@ -829,16 +1044,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D16" t="n">
-        <v>346.87</v>
+        <v>571.35</v>
       </c>
       <c r="E16" t="n">
-        <v>19.04</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="17">
@@ -851,374 +1066,380 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>38.99</v>
+        <v>195.13</v>
       </c>
       <c r="E18" t="n">
-        <v>10.26</v>
+        <v>154.56</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>94</v>
+        <v>38.99</v>
       </c>
       <c r="E19" t="n">
-        <v>5.56</v>
+        <v>10.26</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D20" t="n">
-        <v>123.1</v>
+        <v>193.25</v>
       </c>
       <c r="E20" t="n">
-        <v>9.24</v>
+        <v>11.44</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>12</v>
+      </c>
+      <c r="C21" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" t="n">
+        <v>399.79</v>
+      </c>
+      <c r="E21" t="n">
+        <v>11.59</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>3</v>
-      </c>
-      <c r="C22" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" t="n">
-        <v>69.08</v>
-      </c>
-      <c r="E22" t="n">
-        <v>5.56</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>9</v>
       </c>
       <c r="C23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D23" t="n">
-        <v>204.06</v>
+        <v>445.55</v>
       </c>
       <c r="E23" t="n">
-        <v>9.24</v>
+        <v>162.47</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D24" t="n">
-        <v>-17.05</v>
+        <v>313.98</v>
       </c>
       <c r="E24" t="n">
-        <v>10.26</v>
+        <v>15.12</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" t="n">
+        <v>67.63</v>
+      </c>
+      <c r="E25" t="n">
+        <v>10.26</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>10</v>
-      </c>
-      <c r="C26" t="n">
-        <v>7</v>
-      </c>
-      <c r="D26" t="n">
-        <v>169.4</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>86.69</v>
+        <v>52.49</v>
       </c>
       <c r="E27" t="n">
-        <v>25.06</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" t="n">
+        <v>11</v>
+      </c>
+      <c r="D28" t="n">
+        <v>373.2</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>9</v>
+      </c>
+      <c r="C29" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" t="n">
+        <v>401.47</v>
+      </c>
+      <c r="E29" t="n">
+        <v>187.85</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>ETH</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>10.26</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>2</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
-        <v>5.56</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>9.24</v>
+        <v>154.56</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>10.26</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>11.44</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>2</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>6.02</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>5m</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>2</v>
-      </c>
-      <c r="C38" t="n">
-        <v>2</v>
-      </c>
-      <c r="D38" t="n">
-        <v>19.04</v>
+        <v>11.59</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" t="n">
+        <v>99.55</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>10.26</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
-        <v>9.800000000000001</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" t="n">
-        <v>-4.24</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1228,51 +1449,61 @@
         <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>9.24</v>
+        <v>10.26</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-4.24</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C47" t="n">
         <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>5.56</v>
+        <v>9.24</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1282,147 +1513,233 @@
         <v>1</v>
       </c>
       <c r="D48" t="n">
-        <v>9.24</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D49" t="n">
-        <v>10.26</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>154.56</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>5.88</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>2</v>
-      </c>
-      <c r="C52" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" t="n">
-        <v>5.56</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D53" t="n">
-        <v>9.24</v>
+        <v>162.47</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="n">
+        <v>15.12</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
         <v>10.26</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>3</v>
-      </c>
-      <c r="C57" t="n">
-        <v>2</v>
-      </c>
-      <c r="D57" t="n">
-        <v>15.82</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" t="n">
+        <v>3</v>
+      </c>
+      <c r="D58" t="n">
+        <v>90.47</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>4</v>
+      </c>
+      <c r="C59" t="n">
+        <v>4</v>
+      </c>
+      <c r="D59" t="n">
+        <v>87.12</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>10.26</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D63" t="n">
+        <v>18.17</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B58" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" t="n">
-        <v>9.24</v>
+      <c r="B64" t="n">
+        <v>5</v>
+      </c>
+      <c r="C64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D64" t="n">
+        <v>169.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-22 23:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-22.xlsx
+++ b/reports/2026-09-22.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -859,6 +859,135 @@
       </c>
       <c r="K10" t="n">
         <v>5.88</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-22T21:11:39.551993+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-0.00102</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:14:11.057144+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F12" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="G12" t="n">
+        <v>23</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.789</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.00128</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>11.27</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-22T23:26:28.210148+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-0.00123</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1.91</v>
       </c>
     </row>
   </sheetData>
@@ -872,7 +1001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -894,7 +1023,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -904,7 +1033,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -924,7 +1053,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.9166666666666666</v>
       </c>
     </row>
     <row r="6">
@@ -934,7 +1063,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>187.85</v>
+        <v>203.33</v>
       </c>
     </row>
     <row r="7">
@@ -944,7 +1073,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>192.09</v>
+        <v>207.57</v>
       </c>
     </row>
     <row r="8">
@@ -964,7 +1093,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>45.3</v>
+        <v>48.96</v>
       </c>
     </row>
     <row r="10">
@@ -974,7 +1103,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1592.23</v>
+        <v>1607.71</v>
       </c>
     </row>
     <row r="12">
@@ -1025,16 +1154,16 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>18</v>
+      </c>
+      <c r="C15" t="n">
         <v>14</v>
       </c>
-      <c r="C15" t="n">
-        <v>10</v>
-      </c>
       <c r="D15" t="n">
-        <v>255.81</v>
+        <v>459.31</v>
       </c>
       <c r="E15" t="n">
-        <v>99.55</v>
+        <v>103.76</v>
       </c>
     </row>
     <row r="16">
@@ -1044,16 +1173,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D16" t="n">
-        <v>571.35</v>
+        <v>734.13</v>
       </c>
       <c r="E16" t="n">
-        <v>88.3</v>
+        <v>99.56999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -1108,16 +1237,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>193.25</v>
+        <v>260.66</v>
       </c>
       <c r="E20" t="n">
-        <v>11.44</v>
+        <v>13.74</v>
       </c>
     </row>
     <row r="21">
@@ -1127,16 +1256,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D21" t="n">
-        <v>399.79</v>
+        <v>698.66</v>
       </c>
       <c r="E21" t="n">
-        <v>11.59</v>
+        <v>24.77</v>
       </c>
     </row>
     <row r="22">
@@ -1153,16 +1282,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C23" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D23" t="n">
-        <v>445.55</v>
+        <v>580.55</v>
       </c>
       <c r="E23" t="n">
-        <v>162.47</v>
+        <v>176.04</v>
       </c>
     </row>
     <row r="24">
@@ -1172,13 +1301,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D24" t="n">
-        <v>313.98</v>
+        <v>362.56</v>
       </c>
       <c r="E24" t="n">
         <v>15.12</v>
@@ -1191,16 +1320,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D25" t="n">
-        <v>67.63</v>
+        <v>250.33</v>
       </c>
       <c r="E25" t="n">
-        <v>10.26</v>
+        <v>12.17</v>
       </c>
     </row>
     <row r="26">
@@ -1236,13 +1365,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C28" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D28" t="n">
-        <v>373.2</v>
+        <v>552.78</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1255,16 +1384,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C29" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D29" t="n">
-        <v>401.47</v>
+        <v>588.17</v>
       </c>
       <c r="E29" t="n">
-        <v>187.85</v>
+        <v>203.33</v>
       </c>
     </row>
     <row r="31">
@@ -1335,13 +1464,13 @@
         </is>
       </c>
       <c r="B36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" t="n">
         <v>3</v>
       </c>
-      <c r="C36" t="n">
-        <v>2</v>
-      </c>
       <c r="D36" t="n">
-        <v>11.44</v>
+        <v>13.74</v>
       </c>
     </row>
     <row r="37">
@@ -1351,13 +1480,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>11.59</v>
+        <v>24.77</v>
       </c>
     </row>
     <row r="39">
@@ -1389,13 +1518,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D40" t="n">
-        <v>99.55</v>
+        <v>103.76</v>
       </c>
     </row>
     <row r="41">
@@ -1405,13 +1534,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D41" t="n">
-        <v>88.3</v>
+        <v>99.56999999999999</v>
       </c>
     </row>
     <row r="43">
@@ -1548,198 +1677,246 @@
         <v>5.88</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>11.27</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C53" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>162.47</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>2</v>
-      </c>
-      <c r="C54" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" t="n">
-        <v>15.12</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" t="n">
-        <v>10.26</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>8</v>
+      </c>
+      <c r="C56" t="n">
+        <v>7</v>
+      </c>
+      <c r="D56" t="n">
+        <v>176.04</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="n">
+        <v>15.12</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D58" t="n">
-        <v>90.47</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>4</v>
-      </c>
-      <c r="C59" t="n">
-        <v>4</v>
-      </c>
-      <c r="D59" t="n">
-        <v>87.12</v>
+        <v>12.17</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>1</v>
-      </c>
-      <c r="C60" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" t="n">
-        <v>10.26</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>5</v>
+      </c>
+      <c r="C61" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" t="n">
+        <v>92.77</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>6</v>
+      </c>
+      <c r="C62" t="n">
+        <v>6</v>
+      </c>
+      <c r="D62" t="n">
+        <v>100.3</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="n">
+        <v>10.26</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C63" t="n">
-        <v>3</v>
-      </c>
-      <c r="D63" t="n">
-        <v>18.17</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="B66" t="n">
+        <v>6</v>
+      </c>
+      <c r="C66" t="n">
+        <v>5</v>
+      </c>
+      <c r="D66" t="n">
+        <v>22.38</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B64" t="n">
-        <v>5</v>
-      </c>
-      <c r="C64" t="n">
-        <v>5</v>
-      </c>
-      <c r="D64" t="n">
-        <v>169.68</v>
+      <c r="B67" t="n">
+        <v>6</v>
+      </c>
+      <c r="C67" t="n">
+        <v>6</v>
+      </c>
+      <c r="D67" t="n">
+        <v>180.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>